<commit_message>
v1.4a: simulated supplier names across Projects 01-06
All 17 suppliers renamed to simulated names that state their function
(CloudCo, CodeCo, OfficeCo, ChatCo, PaymentsCo and others) in Markdown,
CSV, workbooks, Word and PDF files. Stand-in disclosure sentences removed;
one Simulated case study line kept per page. Workbooks recalculated:
0 formula errors, no numeric change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQeRkTQscLLdPxf8AsP1RD
</commit_message>
<xml_diff>
--- a/02-risk-register/02-master-risk-register.xlsx
+++ b/02-risk-register/02-master-risk-register.xlsx
@@ -169,13 +169,13 @@
     <t xml:space="preserve">PUBLISHING</t>
   </si>
   <si>
-    <t xml:space="preserve">GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload this .xlsx next to its .md file. GitHub cannot preview .xlsx, so the project README links to it as a download.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notion</t>
+    <t xml:space="preserve">CodeCo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload this .xlsx next to its .md file. CodeCo cannot preview .xlsx, so the project README links to it as a download.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WikiCo</t>
   </si>
   <si>
     <t xml:space="preserve">Import the matching CSV files from the data/ folder (Settings → Import → CSV) for sortable databases.</t>
@@ -550,13 +550,13 @@
     <t xml:space="preserve">R-001</t>
   </si>
   <si>
-    <t xml:space="preserve">Google Workspace, Slack and GitHub user accounts (Confidential data). Vulnerability: human susceptibility to credential-harvesting, compounded by relay-able authenticator-app one-time codes on standard accounts and only 60% policy acknowledgement recorded in CGI-TRK-001.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An external financially motivated attacker sends a credential-harvesting email impersonating Google Workspace to Cypher Group personnel; a user enters their password and one-time code into an attacker-in-the-middle proxy, resulting in session takeover of a corporate account, leading to unauthorised access to Confidential customer correspondence, business email compromise against Finance, and attempted lateral movement toward GitHub and AWS.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CGI-POL-002 §4.3.1 MFA mandated on Google Workspace, Slack, GitHub, AWS, Stripe and the production database; CGI-POL-002 §4.3.3 phishing-resistant FIDO2/WebAuthn or device-bound passkey mandated for all privileged accounts; CGI-POL-002 §4.3.4 passkey-first factor preference for standard accounts; CGI-POL-002 §4.3.5 SMS and voice prohibited as MFA factors; CGI-POL-002 §4.3.7 unsolicited MFA prompts reportable within one hour; CGI-POL-002 §4.1.5 and §4.1.6 password uniqueness and breach-list screening; CGI-POL-002 §4.2.1 credentials held only in the password manager; CGI-POL-002 §4.6.1 SSO through Google Workspace to centralise revocation; CGI-POL-002 §4.6.2 lockout after 10 failed attempts; CGI-POL-001 §4.7.3 suspected phishing forwarded, not interacted with; CGI-POL-001 §4.3.1 credential sharing prohibited; CGI-POL-003 §4.3.6 security awareness induction within 10 business days; CGI-POL-005 §5.2.2 one-hour reporting obligation; CGI-POL-005 §5.4 SEV2 acknowledgement within 30 minutes and containment within 8 hours.</t>
+    <t xml:space="preserve">OfficeCo, ChatCo and CodeCo user accounts (Confidential data). Vulnerability: human susceptibility to credential-harvesting, compounded by relay-able authenticator-app one-time codes on standard accounts and only 60% policy acknowledgement recorded in CGI-TRK-001.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An external financially motivated attacker sends a credential-harvesting email impersonating OfficeCo to Cypher Group personnel; a user enters their password and one-time code into an attacker-in-the-middle proxy, resulting in session takeover of a corporate account, leading to unauthorised access to Confidential customer correspondence, business email compromise against Finance, and attempted lateral movement toward CodeCo and CloudCo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI-POL-002 §4.3.1 MFA mandated on OfficeCo, ChatCo, CodeCo, CloudCo, PaymentsCo and the production database; CGI-POL-002 §4.3.3 phishing-resistant FIDO2/WebAuthn or device-bound passkey mandated for all privileged accounts; CGI-POL-002 §4.3.4 passkey-first factor preference for standard accounts; CGI-POL-002 §4.3.5 SMS and voice prohibited as MFA factors; CGI-POL-002 §4.3.7 unsolicited MFA prompts reportable within one hour; CGI-POL-002 §4.1.5 and §4.1.6 password uniqueness and breach-list screening; CGI-POL-002 §4.2.1 credentials held only in the password manager; CGI-POL-002 §4.6.1 SSO through OfficeCo to centralise revocation; CGI-POL-002 §4.6.2 lockout after 10 failed attempts; CGI-POL-001 §4.7.3 suspected phishing forwarded, not interacted with; CGI-POL-001 §4.3.1 credential sharing prohibited; CGI-POL-003 §4.3.6 security awareness induction within 10 business days; CGI-POL-005 §5.2.2 one-hour reporting obligation; CGI-POL-005 §5.4 SEV2 acknowledgement within 30 minutes and containment within 8 hours.</t>
   </si>
   <si>
     <t xml:space="preserve">IT Operations Manager</t>
@@ -571,7 +571,7 @@
     <t xml:space="preserve">A ransomware affiliate delivers a loader through a malicious document or a drive-by exploit against an unpatched browser on a Cypher Group workstation, resulting in encryption of local and synchronised corporate data and attempted enumeration of reachable network shares and cloud storage, leading to loss of working data, extortion demand, service degradation for approximately 200 SMB customers and an unquantified recovery time because no restore has ever been tested.</t>
   </si>
   <si>
-    <t xml:space="preserve">CGI-POL-001 §4.4.3 operating system and browser security updates applied within 14 calendar days of release; CGI-POL-001 §4.4.1 full-disk encryption mandatory on every device; CGI-POL-001 §4.4.2 automatic screen lock at 10 minutes; CGI-POL-001 §4.4.4 jailbroken or rooted devices prohibited; CGI-POL-001 §4.2.3 prohibition on disabling endpoint protection, disk encryption or logging; CGI-POL-001 §4.6.2 prohibition on unlicensed or untrusted software; CGI-POL-002 §4.4.1 separate administrative accounts, not used for email or browsing, so an infected user session holds no infrastructure rights; CGI-POL-003 §4.1.1 least privilege and §4.2.1 role profiles excluding Engineering from AWS production; CGI-POL-004 §4.2 encryption at rest required for Confidential and Restricted data; CGI-POL-005 §5.4 SEV1 acknowledgement within 15 minutes and containment within 4 hours; CGI-POL-005 §5.5 defined contain, eradicate and recover sequence with a timestamped decision log.</t>
+    <t xml:space="preserve">CGI-POL-001 §4.4.3 operating system and browser security updates applied within 14 calendar days of release; CGI-POL-001 §4.4.1 full-disk encryption mandatory on every device; CGI-POL-001 §4.4.2 automatic screen lock at 10 minutes; CGI-POL-001 §4.4.4 jailbroken or rooted devices prohibited; CGI-POL-001 §4.2.3 prohibition on disabling endpoint protection, disk encryption or logging; CGI-POL-001 §4.6.2 prohibition on unlicensed or untrusted software; CGI-POL-002 §4.4.1 separate administrative accounts, not used for email or browsing, so an infected user session holds no infrastructure rights; CGI-POL-003 §4.1.1 least privilege and §4.2.1 role profiles excluding Engineering from CloudCo production; CGI-POL-004 §4.2 encryption at rest required for Confidential and Restricted data; CGI-POL-005 §5.4 SEV1 acknowledgement within 15 minutes and containment within 4 hours; CGI-POL-005 §5.5 defined contain, eradicate and recover sequence with a timestamped decision log.</t>
   </si>
   <si>
     <t xml:space="preserve">Mitigate + Transfer</t>
@@ -586,7 +586,7 @@
     <t xml:space="preserve">A departing employee, acting on commercial motive before their effective leaving date, uses their legitimate role-profile access to export customer account records and internal documentation to a personal cloud storage account and a removable drive, resulting in unauthorised extraction of Restricted aggregated personal data, leading to a notifiable personal data breach under GDPR Article 33, contractual breach with affected customers, and potential competitive harm.</t>
   </si>
   <si>
-    <t xml:space="preserve">CGI-POL-003 §4.5.1 immediate notification to IT and the CTO on resignation or termination decision; CGI-POL-003 §4.5.2 all access revoked within four hours of the effective termination time; CGI-POL-003 §4.5.3 involuntary terminations revoked simultaneously with the notification meeting; CGI-POL-003 §4.5.4 shared credentials rotated within four hours; CGI-POL-003 §4.5.5 API keys, deploy keys and personal access tokens rotated within five business days; CGI-POL-003 §4.5.6 accounts suspended and preserved for 90 days rather than deleted, protecting investigative evidence; CGI-POL-003 §4.5.9 mandatory evidenced offboarding checklist; CGI-POL-003 §4.7.1 quarterly privileged access review and §4.7.3 monthly orphaned account reconciliation; CGI-POL-003 §4.1.1 and §4.1.2 least privilege and need to know; CGI-POL-003 §4.2.1 role profiles excluding Sales and Customer Success from source code, AWS and Stripe; CGI-POL-001 §4.11.2 prohibition on transferring company information to personal accounts or storage at any time; CGI-POL-001 §4.8.1 removable media prohibited for Confidential and Restricted data without written CTO approval; CGI-POL-001 §4.10 monitoring notice, which is the legal basis that makes authentication and file-access monitoring usable as a detective control; CGI-POL-004 §4.2 Handling Matrix, prohibiting Restricted data on removable media outright and requiring data owner plus CTO approval for external sharing; CGI-POL-004 §4.1.3 aggregation rule reclassifying a bulk customer export as Restricted.</t>
+    <t xml:space="preserve">CGI-POL-003 §4.5.1 immediate notification to IT and the CTO on resignation or termination decision; CGI-POL-003 §4.5.2 all access revoked within four hours of the effective termination time; CGI-POL-003 §4.5.3 involuntary terminations revoked simultaneously with the notification meeting; CGI-POL-003 §4.5.4 shared credentials rotated within four hours; CGI-POL-003 §4.5.5 API keys, deploy keys and personal access tokens rotated within five business days; CGI-POL-003 §4.5.6 accounts suspended and preserved for 90 days rather than deleted, protecting investigative evidence; CGI-POL-003 §4.5.9 mandatory evidenced offboarding checklist; CGI-POL-003 §4.7.1 quarterly privileged access review and §4.7.3 monthly orphaned account reconciliation; CGI-POL-003 §4.1.1 and §4.1.2 least privilege and need to know; CGI-POL-003 §4.2.1 role profiles excluding Sales and Customer Success from source code, CloudCo and PaymentsCo; CGI-POL-001 §4.11.2 prohibition on transferring company information to personal accounts or storage at any time; CGI-POL-001 §4.8.1 removable media prohibited for Confidential and Restricted data without written CTO approval; CGI-POL-001 §4.10 monitoring notice, which is the legal basis that makes authentication and file-access monitoring usable as a detective control; CGI-POL-004 §4.2 Handling Matrix, prohibiting Restricted data on removable media outright and requiring data owner plus CTO approval for external sharing; CGI-POL-004 §4.1.3 aggregation rule reclassifying a bulk customer export as Restricted.</t>
   </si>
   <si>
     <t xml:space="preserve">Head of People and Operations</t>
@@ -604,19 +604,19 @@
     <t xml:space="preserve">An unauthenticated or low-privilege external attacker probes the production API and discovers a broken object-level authorisation flaw allowing customer identifiers to be manipulated across tenant boundaries, resulting in the ability to enumerate and retrieve the account data of customers other than their own, leading to a cross-tenant personal data breach affecting a substantial share of the approximately 200 customer base, mandatory notification under GDPR Articles 33 and 34, and loss of the enterprise deals currently held at security review.</t>
   </si>
   <si>
-    <t xml:space="preserve">CGI-POL-002 §4.5.1 service account credentials and API keys rotated at least every 180 days and immediately on suspected compromise; CGI-POL-002 §4.5.2 GitHub secret scanning and push protection maintained on all repositories; CGI-POL-002 §4.5.3 any committed secret treated as compromised and rotated, not merely removed from history; CGI-POL-002 §4.5.4 service accounts granted minimum permissions with a named human owner; CGI-POL-004 §4.2 encryption in transit required for every classification above Public; CGI-POL-004 §4.1.4 payment card numbers never stored by Cypher Group, limiting the maximum data at risk; CGI-POL-003 §4.2.1 role profiles restricting production database access to on-call Engineering only; CGI-POL-005 §5.1.1 mandatory reporting of unexpected system behaviour, unexplained changes or new accounts; CGI-POL-005 §5.4 SEV1 classification with four-hour containment target; CGI-POL-005 §5.6.3 defined GDPR 72-hour supervisory authority notification path. Assessed as materially insufficient — see control gap CG-02.</t>
+    <t xml:space="preserve">CGI-POL-002 §4.5.1 service account credentials and API keys rotated at least every 180 days and immediately on suspected compromise; CGI-POL-002 §4.5.2 CodeCo secret scanning and push protection maintained on all repositories; CGI-POL-002 §4.5.3 any committed secret treated as compromised and rotated, not merely removed from history; CGI-POL-002 §4.5.4 service accounts granted minimum permissions with a named human owner; CGI-POL-004 §4.2 encryption in transit required for every classification above Public; CGI-POL-004 §4.1.4 payment card numbers never stored by Cypher Group, limiting the maximum data at risk; CGI-POL-003 §4.2.1 role profiles restricting production database access to on-call Engineering only; CGI-POL-005 §5.1.1 mandatory reporting of unexpected system behaviour, unexplained changes or new accounts; CGI-POL-005 §5.4 SEV1 classification with four-hour containment target; CGI-POL-005 §5.6.3 defined GDPR 72-hour supervisory authority notification path. Assessed as materially insufficient — see control gap CG-02.</t>
   </si>
   <si>
     <t xml:space="preserve">R-005</t>
   </si>
   <si>
-    <t xml:space="preserve">AWS production environment: Simple Storage Service (S3) buckets holding customer data exports and backups, security group network rules, and Identity and Access Management (IAM) policies. Vulnerability: the policy pack governs who may change AWS but defines no secure baseline for how it must be configured, and no automated configuration monitoring or drift detection exists (control gap CG-03).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An administrator with legitimate AWS access misconfigures an S3 bucket policy or access control list while troubleshooting, or provisions a new bucket without the account-level public access block, resulting in customer account data and database exports becoming readable from the public internet without authentication, leading to indexed exposure of Restricted aggregated personal data, discovery by a third party or researcher rather than by Cypher Group, notification obligations under GDPR Articles 33 and 34, and severe reputational damage of the category most commonly reported in the technology press.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CGI-POL-004 §4.2 Handling Matrix requiring encryption at rest for Confidential and Restricted data, restricting Restricted data to named approved systems listed by the data owner, and requiring named-individual access approved by the data owner and the CTO; CGI-POL-004 §4.1.3 aggregation rule classifying bulk customer exports as Restricted and therefore subject to the strictest handling row; CGI-POL-002 §4.3.1 MFA mandated on AWS; CGI-POL-002 §4.3.3 phishing-resistant factor mandated for the privileged AWS accounts that can alter bucket policy; CGI-POL-002 §4.4.1 separate administrative accounts; CGI-POL-002 §4.4.3 AWS root protected by hardware MFA, sealed under CTO control, with alerting on any use; CGI-POL-003 §4.2.1 role profiles excluding non-on-call Engineering, Sales, Finance and Customer Success from AWS production; CGI-POL-003 §4.7.1 quarterly privileged access review with evidenced approval or removal decisions; CGI-POL-003 §4.1.5 mandatory ticket for every access change, preserving the audit trail; CGI-POL-001 §4.2.3 prohibition on circumventing or degrading security controls including logging; CGI-POL-005 §5.1.1 mandatory reporting of unexplained configuration change. Preventive coverage only — no detective control exists. See control gap CG-03.</t>
+    <t xml:space="preserve">CloudCo production environment: Simple Storage Service (S3) buckets holding customer data exports and backups, security group network rules, and Identity and Access Management (IAM) policies. Vulnerability: the policy pack governs who may change CloudCo but defines no secure baseline for how it must be configured, and no automated configuration monitoring or drift detection exists (control gap CG-03).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An administrator with legitimate CloudCo access misconfigures an S3 bucket policy or access control list while troubleshooting, or provisions a new bucket without the account-level public access block, resulting in customer account data and database exports becoming readable from the public internet without authentication, leading to indexed exposure of Restricted aggregated personal data, discovery by a third party or researcher rather than by Cypher Group, notification obligations under GDPR Articles 33 and 34, and severe reputational damage of the category most commonly reported in the technology press.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGI-POL-004 §4.2 Handling Matrix requiring encryption at rest for Confidential and Restricted data, restricting Restricted data to named approved systems listed by the data owner, and requiring named-individual access approved by the data owner and the CTO; CGI-POL-004 §4.1.3 aggregation rule classifying bulk customer exports as Restricted and therefore subject to the strictest handling row; CGI-POL-002 §4.3.1 MFA mandated on CloudCo; CGI-POL-002 §4.3.3 phishing-resistant factor mandated for the privileged CloudCo accounts that can alter bucket policy; CGI-POL-002 §4.4.1 separate administrative accounts; CGI-POL-002 §4.4.3 CloudCo root protected by hardware MFA, sealed under CTO control, with alerting on any use; CGI-POL-003 §4.2.1 role profiles excluding non-on-call Engineering, Sales, Finance and Customer Success from CloudCo production; CGI-POL-003 §4.7.1 quarterly privileged access review with evidenced approval or removal decisions; CGI-POL-003 §4.1.5 mandatory ticket for every access change, preserving the audit trail; CGI-POL-001 §4.2.3 prohibition on circumventing or degrading security controls including logging; CGI-POL-005 §5.1.1 mandatory reporting of unexplained configuration change. Preventive coverage only — no detective control exists. See control gap CG-03.</t>
   </si>
   <si>
     <t xml:space="preserve">Inherent</t>
@@ -646,7 +646,7 @@
     <t xml:space="preserve">Likelihood 4 → 3 only. The Project 1 controls address credential-borne API abuse — key rotation, secret scanning, least-privilege service accounts. They do not address authorisation logic defects, which is the actual vulnerability class in this scenario. No policy in the pack requires code review, security testing, dependency scanning or a vulnerability remediation SLA (CG-02). Impact 5 → 4. Encryption in transit, the exclusion of card numbers from Cypher's systems (CGI-POL-004 §4.1.4) and the SEV1 four-hour containment target reduce both the maximum data at risk and the exposure window. This risk remains High after treatment and is the single strongest argument in the register for the next tranche of investment. Recording that honestly is more valuable than manufacturing a green score.</t>
   </si>
   <si>
-    <t xml:space="preserve">Likelihood 4 → 3 only. Quarterly privileged access review (CGI-POL-003 §4.7.1), the role profiles that exclude most of the company from AWS production, and mandatory ticketing (§4.1.5) reduce the number of hands able to cause the misconfiguration and preserve an audit trail. But every one of these is a preventive administrative control acting on people. There is no technical guardrail and no detective control — no account-level S3 Block Public Access enforcement, no AWS Config rules, no drift alerting (CG-03). A misconfiguration made by an authorised administrator would therefore still occur and would not be detected internally. Impact 5 → 4. The encryption-at-rest requirement and the named-approved-systems restriction in CGI-POL-004 §4.2 limit both the readability and the concentration of exposed data.</t>
+    <t xml:space="preserve">Likelihood 4 → 3 only. Quarterly privileged access review (CGI-POL-003 §4.7.1), the role profiles that exclude most of the company from CloudCo production, and mandatory ticketing (§4.1.5) reduce the number of hands able to cause the misconfiguration and preserve an audit trail. But every one of these is a preventive administrative control acting on people. There is no technical guardrail and no detective control — no account-level S3 Block Public Access enforcement, no AWS Config rules, no drift alerting (CG-03). A misconfiguration made by an authorised administrator would therefore still occur and would not be detected internally. Impact 5 → 4. The encryption-at-rest requirement and the named-approved-systems restriction in CGI-POL-004 §4.2 limit both the readability and the concentration of exposed data.</t>
   </si>
   <si>
     <t xml:space="preserve">Treatment ID</t>
@@ -754,7 +754,7 @@
     <t xml:space="preserve">TP-06</t>
   </si>
   <si>
-    <t xml:space="preserve">Enable Google Workspace and endpoint data loss prevention rules for bulk export of Confidential and Restricted data, and add an automated alert on large downloads by any account in a notice period. Closes CG-05.</t>
+    <t xml:space="preserve">Enable OfficeCo and endpoint data loss prevention rules for bulk export of Confidential and Restricted data, and add an automated alert on large downloads by any account in a notice period. Closes CG-05.</t>
   </si>
   <si>
     <t xml:space="preserve">Detective</t>
@@ -781,7 +781,7 @@
     <t xml:space="preserve">TP-09</t>
   </si>
   <si>
-    <t xml:space="preserve">Enable AWS account-level S3 Block Public Access, apply a Service Control Policy preventing its removal, and enable AWS Config rules with alerting for public storage, unencrypted volumes and unrestricted security groups. Closes CG-03.</t>
+    <t xml:space="preserve">Enable CloudCo account-level S3 Block Public Access, apply a Service Control Policy preventing its removal, and enable AWS Config rules with alerting for public storage, unencrypted volumes and unrestricted security groups. Closes CG-03.</t>
   </si>
   <si>
     <t xml:space="preserve">CGI-POL-004 §4.2</t>
@@ -877,7 +877,7 @@
     <t xml:space="preserve">Storage, processing and breach of primary account numbers (payment card data), which would place Cypher Group in PCI DSS scope and raise the maximum credible impact of R-004 and R-005 to score 5.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cypher Group does not store card numbers. All card data is held by Stripe; Cypher retains payment metadata only. The activity that would create the risk is not performed.</t>
+    <t xml:space="preserve">Cypher Group does not store card numbers. All card data is held by PaymentsCo; Cypher retains payment metadata only. The activity that would create the risk is not performed.</t>
   </si>
   <si>
     <t xml:space="preserve">CGI-POL-004 §4.1.4</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">KRI-05</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of AWS resources failing the configuration baseline</t>
+    <t xml:space="preserve">Number of CloudCo resources failing the configuration baseline</t>
   </si>
   <si>
     <t xml:space="preserve">AWS Config (TP-09)</t>
@@ -1852,208 +1852,306 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CGI-RSK-001 — Master Information Security Risk Register v1.0</t>
+        </is>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SIMULATED CASE STUDY. Cypher Group Inc. is a simulated company. All risks, scores, costs, names and approvals are invented for a GRC portfolio case study. No certification or attestation is claimed.</t>
+        </is>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>3</v>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Method</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIST SP 800-30 Rev. 1, semi-quantitative 5 × 5. Risk score = Likelihood × Impact, calculated inherent and residual.</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>5</v>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Register owner</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priya Raman, Chief Technology Officer</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>7</v>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prepared by</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O.S, GRC Analyst (engaged)</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>9</v>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approved by</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jerry Olugboye, Chief Executive Officer — 08 September 2026</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>11</v>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-references</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every mitigating control cites a clause in CGI-POL-001 to CGI-POL-005 (Project 01).</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>13</v>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I score the control that is operating, not the control that is written.</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>14</v>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHEETS</t>
+        </is>
       </c>
       <c r="B11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>16</v>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">01_Scales</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anchored likelihood and impact scales, rating thresholds and treatment definitions.</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>18</v>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02_Register</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The register. Columns A–L are the mandated 12 columns in the required order; M–P are governance columns added after them. Scores and ratings are formulas.</t>
+        </is>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>20</v>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03_Residual_Rationale</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why each residual score is what it is.</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>22</v>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">04_Treatment_Plan</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-01 to TP-10 with cost, owner and target residual. Totals are formulas.</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>24</v>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05_Accept_Avoid</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ACC-001 formal acceptance and AVD-001 avoidance by design.</t>
+        </is>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>26</v>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06_Control_Gaps</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CG-01 to CG-05 — what the policy pack does not cover.</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>28</v>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07_KRIs</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seven key risk indicators with green / amber / red thresholds.</t>
+        </is>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>30</v>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08_Summary</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Register summary — every figure is a formula over 02_Register and 04_Treatment_Plan.</t>
+        </is>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>32</v>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09_Issue_Checklist</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quality checks performed before issue.</t>
+        </is>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>33</v>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COLOUR LEGEND</t>
+        </is>
       </c>
       <c r="B22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>35</v>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yellow cell</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input — type or choose here</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>37</v>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grey cell</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formula — do not overwrite</t>
+        </is>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>39</v>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Green</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass / compliant / low</t>
+        </is>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>41</v>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amber</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial / condition / medium</t>
+        </is>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>43</v>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Red</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail / non-compliant / high or critical</t>
+        </is>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>44</v>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUBLISHING</t>
+        </is>
       </c>
       <c r="B29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>46</v>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GitHub</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload this .xlsx next to its .md file. GitHub cannot preview .xlsx, so the project README links to it as a download.</t>
+        </is>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>48</v>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notion</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import the matching CSV files from the data/ folder (Settings → Import → CSV) for sortable databases.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>